<commit_message>
Resolved conflicts in whole project
</commit_message>
<xml_diff>
--- a/src/test-data/AddParticipant.xlsx
+++ b/src/test-data/AddParticipant.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Waveinit_LMS_Playwright_Project_Main\src\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{070EA84F-4E58-47E0-B712-A3EA740B7BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36BBC4C6-85BC-4234-A806-4EF54DC6E0F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="25">
   <si>
     <t>TestCase</t>
   </si>
@@ -93,16 +93,13 @@
     <t xml:space="preserve">Dummy </t>
   </si>
   <si>
-    <t>dummy@test.com</t>
-  </si>
-  <si>
     <t>dummy005@test.com</t>
   </si>
   <si>
-    <t>Admin@124</t>
-  </si>
-  <si>
     <t>dummy007@test.com</t>
+  </si>
+  <si>
+    <t>dummy.com</t>
   </si>
 </sst>
 </file>
@@ -533,7 +530,7 @@
         <v>21</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D5" t="s">
         <v>12</v>
@@ -553,14 +550,12 @@
         <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -570,13 +565,13 @@
         <v>21</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D7" t="s">
         <v>10</v>
       </c>
       <c r="E7">
-        <v>9090909096</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -585,7 +580,7 @@
     <hyperlink ref="C2" r:id="rId1" xr:uid="{8DC5666B-E518-4DB7-B34D-4CF5028411DC}"/>
     <hyperlink ref="C3" r:id="rId2" xr:uid="{D9735392-ED08-4E2E-BE81-394A84F6DDB7}"/>
     <hyperlink ref="F3" r:id="rId3" xr:uid="{1A53E2EC-08CE-43FF-9C07-20340FA5DEFA}"/>
-    <hyperlink ref="C5" r:id="rId4" xr:uid="{0DE61969-FC8D-4953-9FFF-4BFD39F5D88D}"/>
+    <hyperlink ref="C5" r:id="rId4" display="dummy@test.com" xr:uid="{0DE61969-FC8D-4953-9FFF-4BFD39F5D88D}"/>
     <hyperlink ref="C7" r:id="rId5" xr:uid="{B7605E3F-7A62-47A9-B58E-B15E97098A4C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>